<commit_message>
Add director-level candidates for ATM systems project director role
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JmMXk4GVdXerQikF6zQVcP
</commit_message>
<xml_diff>
--- a/sourcing/2026-10-09-giam-doc-du-an-thiet-bi-quan-ly-bay-hn/ung-vien-giam-doc-du-an-thiet-bi-quan-ly-bay-hn.xlsx
+++ b/sourcing/2026-10-09-giam-doc-du-an-thiet-bi-quan-ly-bay-hn/ung-vien-giam-doc-du-an-thiet-bi-quan-ly-bay-hn.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ứng viên'!$A$1:$U$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ứng viên'!$A$1:$U$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -496,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -650,12 +650,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Managing Director; Account Manager (aviation)</t>
+          <t>Managing Director (M8group); nguyên VP Sales &amp; Marketing SIB Group; nguyên GM Kỹ thuật An toàn Chất lượng Bamboo Airways</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>M8group; TAESCO</t>
+          <t>M8group; TAESCO (Account Manager mảng hàng không)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Business Development (Project Manager)</t>
+          <t>BD Project Manager; nguyên Giám đốc Khối Kinh doanh PCC (2017–2022)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -822,37 +822,37 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>QLB-003</t>
+          <t>QLB-004</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Xuan Truong Nguyen</t>
+          <t>Nguyen The Anh</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Aviation Professional</t>
+          <t>Sales Director</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>VATM – Trung tâm Huấn luyện Quản lý bay</t>
+          <t>VIET UY JSC</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Chưa xác minh</t>
+          <t>Hanoi Capital Region</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Làm việc tại Tổng công ty Quản lý bay Việt Nam (VATM) – hiểu khách hàng chính trong JD</t>
+          <t>Sales Director; tốt nghiệp ĐH Bách khoa Hà Nội. Hồ sơ được Google trả về cho truy vấn Sales Director + radar/ATM/quản lý bay tại Hà Nội</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>confirmed</t>
+          <t>probable</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
@@ -862,25 +862,25 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Headline LinkedIn: "Aviation Professional Seeking New Opportunities"</t>
+          <t>Headline LinkedIn: "Willing to take new challanges"</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/xuan-truong-nguyen-8998ab186</t>
+          <t>https://vn.linkedin.com/in/nguyen-the-anh-b9b0b460</t>
         </is>
       </c>
       <c r="M4" s="2" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Chưa thấy kinh nghiệm kinh doanh/đấu thầu; Chức danh và số năm kinh nghiệm chưa rõ; Ngày tín hiệu không rõ</t>
+          <t>Chưa xác minh ngành của VIET UY JSC và kinh nghiệm thiết bị hàng không; Ngày tín hiệu không rõ</t>
         </is>
       </c>
       <c r="O4" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/xuan-truong-nguyen-8998ab186</t>
+          <t>https://vn.linkedin.com/in/nguyen-the-anh-b9b0b460</t>
         </is>
       </c>
       <c r="P4" s="4" t="inlineStr">
@@ -908,60 +908,70 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Theo dõi</t>
+          <t>Chính</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>QLB-W01</t>
+          <t>QLB-003</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Bui Ngoc Toan</t>
+          <t>Xuan Truong Nguyen</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Regional Sales Manager SEA</t>
+          <t>Aviation Professional</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>KISTERS Group</t>
+          <t>VATM – Trung tâm Huấn luyện Quản lý bay</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Chưa xác minh</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Nguyên International BD Manager / Bids &amp; Project Manager tại đối tác công nghiệp chủ chốt của Thales (Aviation – Aerospace – Security) 2020–2024 – sát JD nhất</t>
+          <t>Làm việc tại Tổng công ty Quản lý bay Việt Nam (VATM) – hiểu khách hàng chính trong JD</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>unverified</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr"/>
+          <t>confirmed</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>không rõ</t>
+        </is>
+      </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Chưa thấy tín hiệu tìm việc công khai</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="n"/>
+          <t>Headline LinkedIn: "Aviation Professional Seeking New Opportunities"</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/xuan-truong-nguyen-8998ab186</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>52</v>
+      </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Cần hỏi trực tiếp nhu cầu chuyển việc</t>
+          <t>Cấp bậc chưa rõ – có thể chưa đạt cấp Giám đốc; Chưa thấy kinh nghiệm kinh doanh/đấu thầu; Chức danh và số năm kinh nghiệm chưa rõ; Ngày tín hiệu không rõ</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/bui-ngoc-toan-589053162</t>
+          <t>https://vn.linkedin.com/in/xuan-truong-nguyen-8998ab186</t>
         </is>
       </c>
       <c r="P5" s="4" t="inlineStr">
@@ -994,32 +1004,32 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>QLB-W02</t>
+          <t>QLB-D01</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Cuong Tran</t>
+          <t>Raúl Hernández Verjillo</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Project Development Manager</t>
+          <t>Managing Director Vietnam/South Korea</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Viettel Aerospace (Viettel Manufacturing)</t>
+          <t>Indra (hãng thiết bị ATM/radar lớn)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Vietnam</t>
+          <t>Hanoi Capital Region</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Deputy Head of BD Aviation Products &amp; Maintenance JSC; Sales Team Lead VAECO (2019–2023)</t>
+          <t>[Cấp Director] Defense | Business Development Director | Country Manager APAC – đúng ngành thiết bị quản lý bay; người nước ngoài, có thể vượt mức ngân sách</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -1042,7 +1052,7 @@
       </c>
       <c r="O6" s="3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/cuong-tran-1a282375</t>
+          <t>https://vn.linkedin.com/in/raul-hernandez-verjillo/en</t>
         </is>
       </c>
       <c r="P6" s="4" t="inlineStr">
@@ -1075,32 +1085,32 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>QLB-W03</t>
+          <t>QLB-D02</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Khanh Vu</t>
+          <t>Tuan Tran Duc</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Business Development Manager</t>
+          <t>Business Development Director – Vietnam Gov &amp; Defense</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>SITA</t>
+          <t>(chưa rõ)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Hanoi Capital Region</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Bán giải pháp công nghệ cho sân bay, hãng bay</t>
+          <t>[Cấp Director] BD Director cho khách hàng Chính phủ &amp; Quốc phòng; chuyên gia đo lường, quang điện tử</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -1123,7 +1133,7 @@
       </c>
       <c r="O7" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/khanhnamvu</t>
+          <t>https://vn.linkedin.com/in/tuan-tran-duc-67583b26</t>
         </is>
       </c>
       <c r="P7" s="4" t="inlineStr">
@@ -1156,32 +1166,32 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>QLB-W04</t>
+          <t>QLB-D03</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Hai Bui</t>
+          <t>Lucie Nguyen</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>General Manager Business Development</t>
+          <t>Regional Sales Director</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Vietnam Airlines Engineering (VAECO)</t>
+          <t>Global Airtech</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Vietnam</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Phát triển kinh doanh kỹ thuật hàng không từ 2013</t>
+          <t>[Cấp Director] Nguyên Director Group Commercial APAC – HAECO (12/2023); Corporate Sales Manager Lufthansa – ngành hàng không</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -1204,7 +1214,7 @@
       </c>
       <c r="O8" s="3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/hai-bui-154523172</t>
+          <t>https://vn.linkedin.com/in/lucienguyen1610</t>
         </is>
       </c>
       <c r="P8" s="4" t="inlineStr">
@@ -1237,22 +1247,22 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>QLB-W05</t>
+          <t>QLB-D04</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Ahmed Khadhraoui</t>
+          <t>BIEN Vu ngoc</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Project Manager</t>
+          <t>Director of Business Development</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Artelia Vietnam</t>
+          <t>Thales Cyber and Digital</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1262,7 +1272,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Systems interface &amp; integration manager (Dorsch/DC Asia, dự án sân bay); nguyên Phó phòng khai thác sân bay OACA Tunisia</t>
+          <t>[Cấp Director] Country Leadership Executive; BD Director Telecom, Banking &amp; Technology tại Thales (không phải mảng ATM)</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -1285,7 +1295,7 @@
       </c>
       <c r="O9" s="3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/khadhraoui-ahmed</t>
+          <t>https://vn.linkedin.com/in/vungocbien</t>
         </is>
       </c>
       <c r="P9" s="4" t="inlineStr">
@@ -1318,32 +1328,32 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>QLB-W06</t>
+          <t>QLB-D05</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Mark Nguyen</t>
+          <t>Trac Van Ky</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Business Development Manager</t>
+          <t>Vice Director, Airborne Radar Center</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Core Practice</t>
+          <t>Viettel Aerospace Institute</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Hanoi Capital Region</t>
+          <t>Chưa xác minh</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>18 năm Aviation Specialist tại ACV (2005–2023)</t>
+          <t>[Cấp Director] Phó giám đốc trung tâm radar – chuyên môn kỹ thuật sâu, chưa thấy kinh nghiệm bán hàng</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1366,7 +1376,7 @@
       </c>
       <c r="O10" s="3" t="inlineStr">
         <is>
-          <t>https://www.linkedin.com/in/mark-nguyen-corepractice</t>
+          <t>https://vn.linkedin.com/in/trac-van-ky-976902105</t>
         </is>
       </c>
       <c r="P10" s="4" t="inlineStr">
@@ -1399,32 +1409,32 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>QLB-W07</t>
+          <t>QLB-W01</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Loc Trinh</t>
+          <t>Bui Ngoc Toan</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Senior System Engineer</t>
+          <t>Regional Sales Manager SEA</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Viet Nam Air Traffic Management Corp (VATM)</t>
+          <t>KISTERS Group</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Chưa xác minh</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Radar Engineer VATM 1997–2005, Senior System Engineer từ 2006 – chuyên môn thiết bị quản lý bay sâu</t>
+          <t>[Cấp Manager – tham khảo] Nguyên International BD Manager / Bids &amp; Project Manager tại đối tác công nghiệp chủ chốt của Thales (Aviation – Aerospace – Security) 2020–2024 – sát JD nhất</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1447,7 +1457,7 @@
       </c>
       <c r="O11" s="3" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/in/loc-trinh-24177097</t>
+          <t>https://www.linkedin.com/in/bui-ngoc-toan-589053162</t>
         </is>
       </c>
       <c r="P11" s="4" t="inlineStr">
@@ -1469,32 +1479,599 @@
       </c>
       <c r="U11" s="4" t="n"/>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>QLB-W08</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Quoc Tuan Nguyen</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Key Account Manager</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Thales</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi Capital Region</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>[Cấp Manager – tham khảo] 15+ năm ngành hàng không, KAM tại Thales (hãng thiết bị ATM hàng đầu) – rất sát chuyên môn</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Chưa thấy tín hiệu tìm việc công khai</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="n"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>Cần hỏi trực tiếp nhu cầu chuyển việc</t>
+        </is>
+      </c>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/quoc-tuan-nguyen-71508aa1</t>
+        </is>
+      </c>
+      <c r="P12" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q12" s="5" t="n"/>
+      <c r="R12" s="4" t="n"/>
+      <c r="S12" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T12" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U12" s="4" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>QLB-W02</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Cuong Tran</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Project Development Manager</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Viettel Aerospace (Viettel Manufacturing)</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Vietnam</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>[Cấp Manager – tham khảo] Deputy Head of BD Aviation Products &amp; Maintenance JSC; Sales Team Lead VAECO (2019–2023)</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Chưa thấy tín hiệu tìm việc công khai</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="n"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>Cần hỏi trực tiếp nhu cầu chuyển việc</t>
+        </is>
+      </c>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/cuong-tran-1a282375</t>
+        </is>
+      </c>
+      <c r="P13" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="n"/>
+      <c r="R13" s="4" t="n"/>
+      <c r="S13" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T13" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U13" s="4" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>QLB-W03</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Khanh Vu</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Business Development Manager</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>SITA</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>[Cấp Manager – tham khảo] Bán giải pháp công nghệ cho sân bay, hãng bay</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Chưa thấy tín hiệu tìm việc công khai</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="n"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>Cần hỏi trực tiếp nhu cầu chuyển việc</t>
+        </is>
+      </c>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/khanhnamvu</t>
+        </is>
+      </c>
+      <c r="P14" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q14" s="5" t="n"/>
+      <c r="R14" s="4" t="n"/>
+      <c r="S14" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T14" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U14" s="4" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>QLB-W04</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Hai Bui</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>General Manager Business Development</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Vietnam Airlines Engineering (VAECO)</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>[Cấp Manager – tham khảo] Phát triển kinh doanh kỹ thuật hàng không từ 2013</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Chưa thấy tín hiệu tìm việc công khai</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="n"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>Cần hỏi trực tiếp nhu cầu chuyển việc</t>
+        </is>
+      </c>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/hai-bui-154523172</t>
+        </is>
+      </c>
+      <c r="P15" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="n"/>
+      <c r="R15" s="4" t="n"/>
+      <c r="S15" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T15" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U15" s="4" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>QLB-W05</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Ahmed Khadhraoui</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Artelia Vietnam</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>[Cấp Manager – tham khảo] Systems interface &amp; integration manager (Dorsch/DC Asia, dự án sân bay); nguyên Phó phòng khai thác sân bay OACA Tunisia</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Chưa thấy tín hiệu tìm việc công khai</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="n"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>Cần hỏi trực tiếp nhu cầu chuyển việc</t>
+        </is>
+      </c>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/khadhraoui-ahmed</t>
+        </is>
+      </c>
+      <c r="P16" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="n"/>
+      <c r="R16" s="4" t="n"/>
+      <c r="S16" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T16" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U16" s="4" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>QLB-W06</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Mark Nguyen</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Business Development Manager</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Core Practice</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi Capital Region</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>[Cấp Manager – tham khảo] 18 năm Aviation Specialist tại ACV (2005–2023)</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Chưa thấy tín hiệu tìm việc công khai</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="n"/>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>Cần hỏi trực tiếp nhu cầu chuyển việc</t>
+        </is>
+      </c>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/mark-nguyen-corepractice</t>
+        </is>
+      </c>
+      <c r="P17" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="n"/>
+      <c r="R17" s="4" t="n"/>
+      <c r="S17" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T17" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U17" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Theo dõi</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>QLB-W07</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Loc Trinh</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Senior System Engineer</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Viet Nam Air Traffic Management Corp (VATM)</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>[Cấp Manager – tham khảo] Radar Engineer VATM 1997–2005, Senior System Engineer từ 2006 – chuyên môn thiết bị quản lý bay sâu</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>unverified</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Chưa thấy tín hiệu tìm việc công khai</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="n"/>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>Cần hỏi trực tiếp nhu cầu chuyển việc</t>
+        </is>
+      </c>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>https://vn.linkedin.com/in/loc-trinh-24177097</t>
+        </is>
+      </c>
+      <c r="P18" s="4" t="inlineStr">
+        <is>
+          <t>Chưa liên hệ</t>
+        </is>
+      </c>
+      <c r="Q18" s="5" t="n"/>
+      <c r="R18" s="4" t="n"/>
+      <c r="S18" s="4" t="inlineStr">
+        <is>
+          <t>Chưa phản hồi</t>
+        </is>
+      </c>
+      <c r="T18" s="4" t="inlineStr">
+        <is>
+          <t>Chưa xác minh</t>
+        </is>
+      </c>
+      <c r="U18" s="4" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U11"/>
-  <conditionalFormatting sqref="P2:P11">
+  <autoFilter ref="A1:U18"/>
+  <conditionalFormatting sqref="P2:P18">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Đã liên hệ"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T2:T11">
+  <conditionalFormatting sqref="T2:T18">
     <cfRule type="cellIs" priority="2" operator="equal" dxfId="0">
       <formula>"Đang tìm việc"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="5">
-    <dataValidation sqref="P2:P11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="P2:P18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Chưa liên hệ,Đã liên hệ,Không liên hệ được"</formula1>
     </dataValidation>
-    <dataValidation sqref="R2:R11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="R2:R18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"LinkedIn InMail,LinkedIn kết nối,Email,Điện thoại/Zalo,Giới thiệu,Khác"</formula1>
     </dataValidation>
-    <dataValidation sqref="S2:S11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="S2:S18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Chưa phản hồi,Quan tâm,Không quan tâm,Hẹn phỏng vấn,Từ chối"</formula1>
     </dataValidation>
-    <dataValidation sqref="T2:T11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="T2:T18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Chưa xác minh,Đang tìm việc,Đang làm việc - mở cơ hội,Đang làm việc - không đổi việc,Đã nhận offer nơi khác"</formula1>
     </dataValidation>
-    <dataValidation sqref="Q2:Q11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThan">
+    <dataValidation sqref="Q2:Q18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="date" operator="greaterThan">
       <formula1>DATE(2020,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -1505,13 +2082,21 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId21"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1549,7 +2134,7 @@
         </is>
       </c>
       <c r="B2" s="6">
-        <f>COUNTA('Ứng viên'!D2:D11)</f>
+        <f>COUNTA('Ứng viên'!D2:D18)</f>
         <v/>
       </c>
     </row>
@@ -1560,7 +2145,7 @@
         </is>
       </c>
       <c r="B3" s="6">
-        <f>COUNTIF('Ứng viên'!B2:B11,"Chính")</f>
+        <f>COUNTIF('Ứng viên'!B2:B18,"Chính")</f>
         <v/>
       </c>
     </row>
@@ -1571,7 +2156,7 @@
         </is>
       </c>
       <c r="B4" s="6">
-        <f>COUNTIF('Ứng viên'!I2:I11,"confirmed")</f>
+        <f>COUNTIF('Ứng viên'!I2:I18,"confirmed")</f>
         <v/>
       </c>
     </row>
@@ -1582,7 +2167,7 @@
         </is>
       </c>
       <c r="B5" s="6">
-        <f>COUNTIF('Ứng viên'!I2:I11,"probable")</f>
+        <f>COUNTIF('Ứng viên'!I2:I18,"probable")</f>
         <v/>
       </c>
     </row>
@@ -1593,7 +2178,7 @@
         </is>
       </c>
       <c r="B6" s="6">
-        <f>COUNTIF('Ứng viên'!B2:B11,"Theo dõi")</f>
+        <f>COUNTIF('Ứng viên'!B2:B18,"Theo dõi")</f>
         <v/>
       </c>
     </row>
@@ -1604,7 +2189,7 @@
         </is>
       </c>
       <c r="B7" s="6">
-        <f>COUNTIF('Ứng viên'!P2:P11,"Đã liên hệ")</f>
+        <f>COUNTIF('Ứng viên'!P2:P18,"Đã liên hệ")</f>
         <v/>
       </c>
     </row>
@@ -1615,7 +2200,7 @@
         </is>
       </c>
       <c r="B8" s="6">
-        <f>COUNTIF('Ứng viên'!P2:P11,"Chưa liên hệ")</f>
+        <f>COUNTIF('Ứng viên'!P2:P18,"Chưa liên hệ")</f>
         <v/>
       </c>
     </row>
@@ -1637,7 +2222,7 @@
         </is>
       </c>
       <c r="B10" s="6">
-        <f>COUNTIF('Ứng viên'!S2:S11,"Quan tâm")</f>
+        <f>COUNTIF('Ứng viên'!S2:S18,"Quan tâm")</f>
         <v/>
       </c>
     </row>
@@ -1648,7 +2233,7 @@
         </is>
       </c>
       <c r="B11" s="6">
-        <f>COUNTIF('Ứng viên'!S2:S11,"Hẹn phỏng vấn")</f>
+        <f>COUNTIF('Ứng viên'!S2:S18,"Hẹn phỏng vấn")</f>
         <v/>
       </c>
     </row>
@@ -1659,7 +2244,7 @@
         </is>
       </c>
       <c r="B12" s="6">
-        <f>COUNTIF('Ứng viên'!T2:T11,"Đang tìm việc")</f>
+        <f>COUNTIF('Ứng viên'!T2:T18,"Đang tìm việc")</f>
         <v/>
       </c>
     </row>
@@ -1670,7 +2255,7 @@
         </is>
       </c>
       <c r="B13" s="6">
-        <f>COUNTIF('Ứng viên'!T2:T11,"Chưa xác minh")</f>
+        <f>COUNTIF('Ứng viên'!T2:T18,"Chưa xác minh")</f>
         <v/>
       </c>
     </row>

</xml_diff>